<commit_message>
Rebrand to Coucou 🇫🇷
Rename site to 'Coucou' (a friendly French 'hi'): update title, brand,
hero, og tags, favicon (C), README and tracker. New URL: /coucou/.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/French_Learning_Tracker.xlsx
+++ b/assets/French_Learning_Tracker.xlsx
@@ -614,14 +614,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Learn French with AI  —  Progress Tracker</t>
+          <t>Coucou  —  French Progress Tracker</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to ektasengar.github.io/learn-french-with-ai  ·  pick your target, log your hours, tick milestones</t>
+          <t>Companion to ektasengar.github.io/coucou  ·  pick your target, log your hours, tick milestones</t>
         </is>
       </c>
     </row>

</xml_diff>